<commit_message>
Edited data loading such that it looks at timestamps and removes duplicates and plots raw ground truth and not window ground truth
</commit_message>
<xml_diff>
--- a/mstraczkiewicz/MStraPlots_RT/Detailed_MStra_RT_Results.xlsx
+++ b/mstraczkiewicz/MStraPlots_RT/Detailed_MStra_RT_Results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="375" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="998" uniqueCount="49">
   <si>
     <t>Subject</t>
   </si>
@@ -149,6 +149,21 @@
   </si>
   <si>
     <t>Standing</t>
+  </si>
+  <si>
+    <t>test5</t>
+  </si>
+  <si>
+    <t>test6</t>
+  </si>
+  <si>
+    <t>test7</t>
+  </si>
+  <si>
+    <t>test8</t>
+  </si>
+  <si>
+    <t>test9</t>
   </si>
 </sst>
 </file>
@@ -197,17 +212,17 @@
   <dimension ref="A1:K89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" customWidth="true"/>
-    <col min="2" max="2" width="9.88671875" customWidth="true"/>
+    <col min="1" max="1" width="7.21875" customWidth="true"/>
+    <col min="2" max="2" width="7" customWidth="true"/>
     <col min="3" max="3" width="5.33203125" customWidth="true"/>
-    <col min="4" max="4" width="14.5546875" customWidth="true"/>
-    <col min="5" max="5" width="13.5546875" customWidth="true"/>
+    <col min="4" max="4" width="12.5546875" customWidth="true"/>
+    <col min="5" max="5" width="12.5546875" customWidth="true"/>
     <col min="6" max="6" width="12.5546875" customWidth="true"/>
-    <col min="7" max="7" width="14.5546875" customWidth="true"/>
+    <col min="7" max="7" width="12.5546875" customWidth="true"/>
     <col min="8" max="8" width="6" customWidth="true"/>
-    <col min="9" max="9" width="7" customWidth="true"/>
-    <col min="10" max="10" width="6" customWidth="true"/>
-    <col min="11" max="11" width="5" customWidth="true"/>
+    <col min="9" max="9" width="6" customWidth="true"/>
+    <col min="10" max="10" width="5" customWidth="true"/>
+    <col min="11" max="11" width="6" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -256,28 +271,28 @@
         <v>8</v>
       </c>
       <c r="D2" s="0">
-        <v>0.92626920147720249</v>
+        <v>0.80866814635637485</v>
       </c>
       <c r="E2" s="0">
-        <v>0.90766766838818802</v>
+        <v>0.74834807537670878</v>
       </c>
       <c r="F2" s="0">
-        <v>0.95169811320754716</v>
+        <v>0.95133333333333336</v>
       </c>
       <c r="G2" s="0">
-        <v>0.86753121667641298</v>
+        <v>0.6167521466028929</v>
       </c>
       <c r="H2" s="0">
-        <v>25220</v>
+        <v>21405</v>
       </c>
       <c r="I2" s="0">
-        <v>39240</v>
+        <v>39440</v>
       </c>
       <c r="J2" s="0">
-        <v>1280</v>
+        <v>1095</v>
       </c>
       <c r="K2" s="0">
-        <v>3851</v>
+        <v>13301</v>
       </c>
     </row>
     <row r="3">
@@ -291,19 +306,19 @@
         <v>9</v>
       </c>
       <c r="D3" s="0">
-        <v>0.93517839950568316</v>
+        <v>0.85830863491979104</v>
       </c>
       <c r="E3" s="0">
-        <v>0.91829526724746879</v>
+        <v>0.82337933433839727</v>
       </c>
       <c r="F3" s="0">
-        <v>0.96940726577437863</v>
+        <v>0.96881091617933723</v>
       </c>
       <c r="G3" s="0">
-        <v>0.87230308661092182</v>
+        <v>0.71591138255884301</v>
       </c>
       <c r="H3" s="0">
-        <v>25350</v>
+        <v>24850</v>
       </c>
       <c r="I3" s="0">
         <v>39730</v>
@@ -312,7 +327,7 @@
         <v>800</v>
       </c>
       <c r="K3" s="0">
-        <v>3711</v>
+        <v>9861</v>
       </c>
     </row>
     <row r="4">
@@ -396,25 +411,25 @@
         <v>8</v>
       </c>
       <c r="D6" s="0">
-        <v>0.78753407915765727</v>
+        <v>0.78784745072232143</v>
       </c>
       <c r="E6" s="0">
-        <v>0.73349056603773588</v>
+        <v>0.7339882121807465</v>
       </c>
       <c r="F6" s="0">
-        <v>0.73754940711462447</v>
+        <v>0.73833992094861656</v>
       </c>
       <c r="G6" s="0">
-        <v>0.72947615324472248</v>
+        <v>0.72968750000000004</v>
       </c>
       <c r="H6" s="0">
-        <v>9330</v>
+        <v>9340</v>
       </c>
       <c r="I6" s="0">
         <v>15801</v>
       </c>
       <c r="J6" s="0">
-        <v>3320</v>
+        <v>3310</v>
       </c>
       <c r="K6" s="0">
         <v>3460</v>
@@ -457,72 +472,72 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="0">
-        <v>0.97560061387441033</v>
+        <v>0.82189900189232312</v>
       </c>
       <c r="E8" s="0">
-        <v>0</v>
+        <v>0.78571428571428581</v>
       </c>
       <c r="F8" s="0">
-        <v>0</v>
+        <v>0.90256410256410258</v>
       </c>
       <c r="G8" s="0">
-        <v>1</v>
+        <v>0.69565217391304346</v>
       </c>
       <c r="H8" s="0">
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="I8" s="0">
-        <v>413841</v>
+        <v>13351</v>
       </c>
       <c r="J8" s="0">
-        <v>10350</v>
+        <v>950</v>
       </c>
       <c r="K8" s="0">
-        <v>0</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="0">
-        <v>0.99233835701370376</v>
+        <v>0.82189900189232312</v>
       </c>
       <c r="E9" s="0">
-        <v>0</v>
+        <v>0.78666666666666663</v>
       </c>
       <c r="F9" s="0">
-        <v>0</v>
+        <v>0.89847715736040612</v>
       </c>
       <c r="G9" s="0">
-        <v>1</v>
+        <v>0.69960474308300391</v>
       </c>
       <c r="H9" s="0">
-        <v>0</v>
+        <v>8850</v>
       </c>
       <c r="I9" s="0">
-        <v>420941</v>
+        <v>13301</v>
       </c>
       <c r="J9" s="0">
-        <v>3250</v>
+        <v>1000</v>
       </c>
       <c r="K9" s="0">
-        <v>0</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="10">
@@ -530,34 +545,34 @@
         <v>1</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="0">
-        <v>0.99200915522501365</v>
+        <v>0.82577077494129236</v>
       </c>
       <c r="E10" s="0">
-        <v>0</v>
+        <v>0.708860759493671</v>
       </c>
       <c r="F10" s="0">
-        <v>0</v>
+        <v>0.7466666666666667</v>
       </c>
       <c r="G10" s="0">
-        <v>1</v>
+        <v>0.67469879518072284</v>
       </c>
       <c r="H10" s="0">
-        <v>0</v>
+        <v>2800</v>
       </c>
       <c r="I10" s="0">
-        <v>347601</v>
+        <v>8101</v>
       </c>
       <c r="J10" s="0">
-        <v>2800</v>
+        <v>950</v>
       </c>
       <c r="K10" s="0">
-        <v>0</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="11">
@@ -565,244 +580,244 @@
         <v>1</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="0">
-        <v>0.99315070447858311</v>
+        <v>0.9090977956215438</v>
       </c>
       <c r="E11" s="0">
-        <v>0</v>
+        <v>0.84615384615384603</v>
       </c>
       <c r="F11" s="0">
-        <v>0</v>
+        <v>0.90410958904109584</v>
       </c>
       <c r="G11" s="0">
-        <v>1</v>
+        <v>0.79518072289156627</v>
       </c>
       <c r="H11" s="0">
-        <v>0</v>
+        <v>3300</v>
       </c>
       <c r="I11" s="0">
-        <v>348001</v>
+        <v>8701</v>
       </c>
       <c r="J11" s="0">
-        <v>2400</v>
+        <v>350</v>
       </c>
       <c r="K11" s="0">
-        <v>0</v>
+        <v>850</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="0">
-        <v>0.83194675540765395</v>
+        <v>0.5808504191495808</v>
       </c>
       <c r="E12" s="0">
-        <v>0.90826521344232514</v>
+        <v>0.27826086956521745</v>
       </c>
       <c r="F12" s="0">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G12" s="0">
-        <v>0.83194675540765395</v>
+        <v>0.19277108433734941</v>
       </c>
       <c r="H12" s="0">
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="I12" s="0">
-        <v>0</v>
+        <v>4951</v>
       </c>
       <c r="J12" s="0">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="K12" s="0">
-        <v>1111</v>
+        <v>3350</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="0">
-        <v>0.82438360308576619</v>
+        <v>0.78790021209978789</v>
       </c>
       <c r="E13" s="0">
-        <v>0.90373932509742139</v>
+        <v>0.73749999999999993</v>
       </c>
       <c r="F13" s="0">
-        <v>1</v>
+        <v>0.76623376623376627</v>
       </c>
       <c r="G13" s="0">
-        <v>0.82438360308576619</v>
+        <v>0.71084337349397586</v>
       </c>
       <c r="H13" s="0">
-        <v>5450</v>
+        <v>2950</v>
       </c>
       <c r="I13" s="0">
-        <v>0</v>
+        <v>4851</v>
       </c>
       <c r="J13" s="0">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="K13" s="0">
-        <v>1161</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="0">
-        <v>0.93938898872733212</v>
+        <v>0.78023588015529999</v>
       </c>
       <c r="E14" s="0">
-        <v>0.96874736753432733</v>
+        <v>0.62500000000000011</v>
       </c>
       <c r="F14" s="0">
-        <v>1</v>
+        <v>0.64935064935064934</v>
       </c>
       <c r="G14" s="0">
-        <v>0.93938898872733212</v>
+        <v>0.60240963855421692</v>
       </c>
       <c r="H14" s="0">
-        <v>5750</v>
+        <v>2500</v>
       </c>
       <c r="I14" s="0">
-        <v>0</v>
+        <v>8151</v>
       </c>
       <c r="J14" s="0">
-        <v>0</v>
+        <v>1350</v>
       </c>
       <c r="K14" s="0">
-        <v>371</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="0">
-        <v>0.94755758862930894</v>
+        <v>0.87180426342392503</v>
       </c>
       <c r="E15" s="0">
-        <v>0.97307272879791962</v>
+        <v>0.7712418300653594</v>
       </c>
       <c r="F15" s="0">
-        <v>1</v>
+        <v>0.84285714285714286</v>
       </c>
       <c r="G15" s="0">
-        <v>0.94755758862930894</v>
+        <v>0.71084337349397586</v>
       </c>
       <c r="H15" s="0">
-        <v>5800</v>
+        <v>2950</v>
       </c>
       <c r="I15" s="0">
-        <v>0</v>
+        <v>8951</v>
       </c>
       <c r="J15" s="0">
-        <v>0</v>
+        <v>550</v>
       </c>
       <c r="K15" s="0">
-        <v>321</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="0">
-        <v>0.89708041102593383</v>
+        <v>0.75231630125676541</v>
       </c>
       <c r="E16" s="0">
-        <v>0.94574843091737604</v>
+        <v>0.7065217391304347</v>
       </c>
       <c r="F16" s="0">
-        <v>1</v>
+        <v>0.64356435643564358</v>
       </c>
       <c r="G16" s="0">
-        <v>0.89708041102593383</v>
+        <v>0.7831325301204819</v>
       </c>
       <c r="H16" s="0">
-        <v>5500</v>
+        <v>3250</v>
       </c>
       <c r="I16" s="0">
-        <v>0</v>
+        <v>4951</v>
       </c>
       <c r="J16" s="0">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="K16" s="0">
-        <v>631</v>
+        <v>900</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C17" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="0">
-        <v>0.78290654053172404</v>
+        <v>0.85140264790297193</v>
       </c>
       <c r="E17" s="0">
-        <v>0.87823620894703147</v>
+        <v>0.7841291190316072</v>
       </c>
       <c r="F17" s="0">
-        <v>1</v>
+        <v>0.85735294117647054</v>
       </c>
       <c r="G17" s="0">
-        <v>0.78290654053172404</v>
+        <v>0.72242874845105332</v>
       </c>
       <c r="H17" s="0">
-        <v>4800</v>
+        <v>2915</v>
       </c>
       <c r="I17" s="0">
-        <v>0</v>
+        <v>6281</v>
       </c>
       <c r="J17" s="0">
-        <v>0</v>
+        <v>485</v>
       </c>
       <c r="K17" s="0">
-        <v>1331</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="18">
@@ -3338,7 +3353,7 @@
     <col min="2" max="2" width="10.88671875" customWidth="true"/>
     <col min="3" max="3" width="13.88671875" customWidth="true"/>
     <col min="4" max="4" width="13.88671875" customWidth="true"/>
-    <col min="5" max="5" width="12.5546875" customWidth="true"/>
+    <col min="5" max="5" width="11.5546875" customWidth="true"/>
     <col min="6" max="6" width="12.5546875" customWidth="true"/>
   </cols>
   <sheetData>
@@ -3367,19 +3382,19 @@
         <v>9</v>
       </c>
       <c r="B2" s="0">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="C2" s="0">
-        <v>0.75331737173246127</v>
+        <v>0.8628186691189097</v>
       </c>
       <c r="D2" s="0">
-        <v>0.88231086236728806</v>
+        <v>0.88626402390431447</v>
       </c>
       <c r="E2" s="0">
-        <v>0.75146397333616166</v>
+        <v>0.75520517800038978</v>
       </c>
       <c r="F2" s="0">
-        <v>0.69074720545812085</v>
+        <v>0.8136431892026792</v>
       </c>
     </row>
     <row r="3">
@@ -3387,19 +3402,19 @@
         <v>8</v>
       </c>
       <c r="B3" s="0">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="C3" s="0">
-        <v>0.7142714410383465</v>
+        <v>0.78609871070904369</v>
       </c>
       <c r="D3" s="0">
-        <v>0.87889065521766474</v>
+        <v>0.76422004231926133</v>
       </c>
       <c r="E3" s="0">
-        <v>0.72029369071359561</v>
+        <v>0.64528677151570457</v>
       </c>
       <c r="F3" s="0">
-        <v>0.65835519672934961</v>
+        <v>0.6884624016777845</v>
       </c>
     </row>
   </sheetData>
@@ -3411,7 +3426,7 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" customWidth="true"/>
+    <col min="1" max="1" width="7" customWidth="true"/>
     <col min="2" max="2" width="10.88671875" customWidth="true"/>
     <col min="3" max="3" width="13.88671875" customWidth="true"/>
     <col min="4" max="4" width="13.88671875" customWidth="true"/>
@@ -3441,162 +3456,162 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="B2" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C2" s="0">
-        <v>0.98827470764792769</v>
+        <v>0.833488390638083</v>
       </c>
       <c r="D2" s="0">
-        <v>0</v>
+        <v>0.9600721247563353</v>
       </c>
       <c r="E2" s="0">
-        <v>1</v>
+        <v>0.66633176458086796</v>
       </c>
       <c r="F2" s="0">
-        <v>0</v>
+        <v>0.78586370485755297</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="B3" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3" s="0">
-        <v>0.99588409614751394</v>
+        <v>0.91414504619129278</v>
       </c>
       <c r="D3" s="0">
-        <v>0.5</v>
+        <v>0.97994124286283357</v>
       </c>
       <c r="E3" s="0">
-        <v>1</v>
+        <v>0.83130656672381487</v>
       </c>
       <c r="F3" s="0">
-        <v>0.5</v>
+        <v>0.89914734476009639</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="B4" s="0">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C4" s="0">
-        <v>0.81580522885452411</v>
+        <v>0.84644793331453105</v>
       </c>
       <c r="D4" s="0">
-        <v>1</v>
+        <v>0.80633471143216262</v>
       </c>
       <c r="E4" s="0">
-        <v>0.81580522885452411</v>
+        <v>0.810546875</v>
       </c>
       <c r="F4" s="0">
-        <v>0.88964494178875875</v>
+        <v>0.8083867559936615</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B5" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5" s="0">
-        <v>0.97932641708013835</v>
+        <v>0.82189900189232312</v>
       </c>
       <c r="D5" s="0">
-        <v>0.5</v>
+        <v>0.90052062996225435</v>
       </c>
       <c r="E5" s="0">
-        <v>1</v>
+        <v>0.69762845849802368</v>
       </c>
       <c r="F5" s="0">
-        <v>0.5</v>
+        <v>0.78619047619047622</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B6" s="0">
         <v>2</v>
       </c>
       <c r="C6" s="0">
-        <v>0.80181965588685711</v>
+        <v>0.86743428528141808</v>
       </c>
       <c r="D6" s="0">
-        <v>0</v>
+        <v>0.82538812785388127</v>
       </c>
       <c r="E6" s="0">
-        <v>1</v>
+        <v>0.73493975903614461</v>
       </c>
       <c r="F6" s="0">
-        <v>0</v>
+        <v>0.77750730282375846</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B7" s="0">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="C7" s="0">
-        <v>0.62848314839494712</v>
+        <v>0.68437531562468434</v>
       </c>
       <c r="D7" s="0">
-        <v>1</v>
+        <v>0.63311688311688319</v>
       </c>
       <c r="E7" s="0">
-        <v>0.62848314839494712</v>
+        <v>0.45180722891566261</v>
       </c>
       <c r="F7" s="0">
-        <v>0.69010871416593056</v>
+        <v>0.50788043478260869</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="B8" s="0">
         <v>2</v>
       </c>
       <c r="C8" s="0">
-        <v>0.93072380049144288</v>
+        <v>0.82602007178961245</v>
       </c>
       <c r="D8" s="0">
-        <v>0.96055268949096284</v>
+        <v>0.74610389610389616</v>
       </c>
       <c r="E8" s="0">
-        <v>0.86991715164366745</v>
+        <v>0.65662650602409633</v>
       </c>
       <c r="F8" s="0">
-        <v>0.91298146781782841</v>
+        <v>0.6981209150326797</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B9" s="0">
         <v>2</v>
       </c>
       <c r="C9" s="0">
-        <v>0.91414504619129278</v>
+        <v>0.80185947457986861</v>
       </c>
       <c r="D9" s="0">
-        <v>0.97994124286283357</v>
+        <v>0.75045864880605706</v>
       </c>
       <c r="E9" s="0">
-        <v>0.83130656672381487</v>
+        <v>0.75278063928576766</v>
       </c>
       <c r="F9" s="0">
-        <v>0.89914734476009639</v>
+        <v>0.74532542908102095</v>
       </c>
     </row>
     <row r="10">
@@ -3628,7 +3643,7 @@
   <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" customWidth="true"/>
+    <col min="1" max="1" width="7.21875" customWidth="true"/>
     <col min="2" max="2" width="10.88671875" customWidth="true"/>
     <col min="3" max="3" width="13.88671875" customWidth="true"/>
     <col min="4" max="4" width="13.88671875" customWidth="true"/>
@@ -3661,19 +3676,19 @@
         <v>2</v>
       </c>
       <c r="B2" s="0">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C2" s="0">
-        <v>0.91405679705874698</v>
+        <v>0.82477582656133741</v>
       </c>
       <c r="D2" s="0">
-        <v>0.63432324241919436</v>
+        <v>0.76763241878070521</v>
       </c>
       <c r="E2" s="0">
-        <v>0.91764473613971853</v>
+        <v>0.73998467343662133</v>
       </c>
       <c r="F2" s="0">
-        <v>0.60562252395053118</v>
+        <v>0.75061103336912061</v>
       </c>
     </row>
     <row r="3">
@@ -3684,16 +3699,16 @@
         <v>10</v>
       </c>
       <c r="C3" s="0">
-        <v>0.91787322120280057</v>
+        <v>0.82426840792556022</v>
       </c>
       <c r="D3" s="0">
-        <v>0.58809878647075942</v>
+        <v>0.85980780171043758</v>
       </c>
       <c r="E3" s="0">
-        <v>0.93026427839201897</v>
+        <v>0.67640275555090279</v>
       </c>
       <c r="F3" s="0">
-        <v>0.55723976653198215</v>
+        <v>0.75131785268289852</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Added energies from QSense to plots and results
</commit_message>
<xml_diff>
--- a/mstraczkiewicz/MStraPlots_RT/Detailed_MStra_RT_Results.xlsx
+++ b/mstraczkiewicz/MStraPlots_RT/Detailed_MStra_RT_Results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="998" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3169" uniqueCount="49">
   <si>
     <t>Subject</t>
   </si>
@@ -222,7 +222,7 @@
     <col min="8" max="8" width="6" customWidth="true"/>
     <col min="9" max="9" width="6" customWidth="true"/>
     <col min="10" max="10" width="5" customWidth="true"/>
-    <col min="11" max="11" width="6" customWidth="true"/>
+    <col min="11" max="11" width="5" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -271,28 +271,28 @@
         <v>8</v>
       </c>
       <c r="D2" s="0">
-        <v>0.80866814635637485</v>
+        <v>0.95912841879995459</v>
       </c>
       <c r="E2" s="0">
-        <v>0.74834807537670878</v>
+        <v>0.94395411395922724</v>
       </c>
       <c r="F2" s="0">
-        <v>0.95133333333333336</v>
+        <v>0.90920770877944324</v>
       </c>
       <c r="G2" s="0">
-        <v>0.6167521466028929</v>
+        <v>0.9814617909481762</v>
       </c>
       <c r="H2" s="0">
-        <v>21405</v>
+        <v>21230</v>
       </c>
       <c r="I2" s="0">
-        <v>39440</v>
+        <v>37930</v>
       </c>
       <c r="J2" s="0">
-        <v>1095</v>
+        <v>2120</v>
       </c>
       <c r="K2" s="0">
-        <v>13301</v>
+        <v>401</v>
       </c>
     </row>
     <row r="3">
@@ -306,28 +306,28 @@
         <v>9</v>
       </c>
       <c r="D3" s="0">
-        <v>0.85830863491979104</v>
+        <v>0.95703776787916606</v>
       </c>
       <c r="E3" s="0">
-        <v>0.82337933433839727</v>
+        <v>0.94863031522700847</v>
       </c>
       <c r="F3" s="0">
-        <v>0.96881091617933723</v>
+        <v>0.93470085470085473</v>
       </c>
       <c r="G3" s="0">
-        <v>0.71591138255884301</v>
+        <v>0.96298122644500017</v>
       </c>
       <c r="H3" s="0">
-        <v>24850</v>
+        <v>27340</v>
       </c>
       <c r="I3" s="0">
-        <v>39730</v>
+        <v>38620</v>
       </c>
       <c r="J3" s="0">
-        <v>800</v>
+        <v>1910</v>
       </c>
       <c r="K3" s="0">
-        <v>9861</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="4">
@@ -341,28 +341,28 @@
         <v>8</v>
       </c>
       <c r="D4" s="0">
-        <v>0.93120171119839201</v>
+        <v>0.93153530819313313</v>
       </c>
       <c r="E4" s="0">
-        <v>0.92100527196121196</v>
+        <v>0.92578070016689784</v>
       </c>
       <c r="F4" s="0">
-        <v>0.98194130925507905</v>
+        <v>0.93387423935091274</v>
       </c>
       <c r="G4" s="0">
-        <v>0.86719030341692915</v>
+        <v>0.91782624297276827</v>
       </c>
       <c r="H4" s="0">
-        <v>21750</v>
+        <v>23020</v>
       </c>
       <c r="I4" s="0">
-        <v>28750</v>
+        <v>27200</v>
       </c>
       <c r="J4" s="0">
-        <v>400</v>
+        <v>1630</v>
       </c>
       <c r="K4" s="0">
-        <v>3331</v>
+        <v>2061</v>
       </c>
     </row>
     <row r="5">
@@ -376,28 +376,28 @@
         <v>9</v>
       </c>
       <c r="D5" s="0">
-        <v>0.89708838118419354</v>
+        <v>0.90389332546430345</v>
       </c>
       <c r="E5" s="0">
-        <v>0.87728941755898071</v>
+        <v>0.89393661842828342</v>
       </c>
       <c r="F5" s="0">
-        <v>0.9779411764705882</v>
+        <v>0.91309771309771315</v>
       </c>
       <c r="G5" s="0">
-        <v>0.79542283003070058</v>
+        <v>0.87556317531198913</v>
       </c>
       <c r="H5" s="0">
-        <v>19950</v>
+        <v>21960</v>
       </c>
       <c r="I5" s="0">
-        <v>28700</v>
+        <v>27050</v>
       </c>
       <c r="J5" s="0">
-        <v>450</v>
+        <v>2090</v>
       </c>
       <c r="K5" s="0">
-        <v>5131</v>
+        <v>3121</v>
       </c>
     </row>
     <row r="6">
@@ -411,28 +411,28 @@
         <v>8</v>
       </c>
       <c r="D6" s="0">
-        <v>0.78784745072232143</v>
+        <v>0.79988080675010198</v>
       </c>
       <c r="E6" s="0">
-        <v>0.7339882121807465</v>
+        <v>0.78387533875338755</v>
       </c>
       <c r="F6" s="0">
-        <v>0.73833992094861656</v>
+        <v>0.6907462686567164</v>
       </c>
       <c r="G6" s="0">
-        <v>0.72968750000000004</v>
+        <v>0.90602975724353951</v>
       </c>
       <c r="H6" s="0">
-        <v>9340</v>
+        <v>11570</v>
       </c>
       <c r="I6" s="0">
-        <v>15801</v>
+        <v>13931</v>
       </c>
       <c r="J6" s="0">
-        <v>3310</v>
+        <v>5180</v>
       </c>
       <c r="K6" s="0">
-        <v>3460</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="7">
@@ -446,28 +446,28 @@
         <v>9</v>
       </c>
       <c r="D7" s="0">
-        <v>0.90504841590674068</v>
+        <v>0.87026417222901198</v>
       </c>
       <c r="E7" s="0">
-        <v>0.88278529980657638</v>
+        <v>0.85966101694915253</v>
       </c>
       <c r="F7" s="0">
-        <v>0.8743295019157088</v>
+        <v>0.75928143712574847</v>
       </c>
       <c r="G7" s="0">
-        <v>0.89140624999999996</v>
+        <v>0.99062499999999998</v>
       </c>
       <c r="H7" s="0">
-        <v>11410</v>
+        <v>12680</v>
       </c>
       <c r="I7" s="0">
-        <v>17471</v>
+        <v>15091</v>
       </c>
       <c r="J7" s="0">
-        <v>1640</v>
+        <v>4020</v>
       </c>
       <c r="K7" s="0">
-        <v>1390</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8">
@@ -481,28 +481,28 @@
         <v>8</v>
       </c>
       <c r="D8" s="0">
-        <v>0.82189900189232312</v>
+        <v>0.87224982256919803</v>
       </c>
       <c r="E8" s="0">
-        <v>0.78571428571428581</v>
+        <v>0.86330935251798557</v>
       </c>
       <c r="F8" s="0">
-        <v>0.90256410256410258</v>
+        <v>0.8605577689243028</v>
       </c>
       <c r="G8" s="0">
-        <v>0.69565217391304346</v>
+        <v>0.8660785886126704</v>
       </c>
       <c r="H8" s="0">
-        <v>8800</v>
+        <v>10800</v>
       </c>
       <c r="I8" s="0">
-        <v>13351</v>
+        <v>12551</v>
       </c>
       <c r="J8" s="0">
-        <v>950</v>
+        <v>1750</v>
       </c>
       <c r="K8" s="0">
-        <v>3850</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="9">
@@ -516,28 +516,28 @@
         <v>9</v>
       </c>
       <c r="D9" s="0">
-        <v>0.82189900189232312</v>
+        <v>0.90265189660960055</v>
       </c>
       <c r="E9" s="0">
-        <v>0.78666666666666663</v>
+        <v>0.89646965489884956</v>
       </c>
       <c r="F9" s="0">
-        <v>0.89847715736040612</v>
+        <v>0.88976377952755903</v>
       </c>
       <c r="G9" s="0">
-        <v>0.69960474308300391</v>
+        <v>0.90327737809752195</v>
       </c>
       <c r="H9" s="0">
-        <v>8850</v>
+        <v>11300</v>
       </c>
       <c r="I9" s="0">
-        <v>13301</v>
+        <v>12901</v>
       </c>
       <c r="J9" s="0">
-        <v>1000</v>
+        <v>1400</v>
       </c>
       <c r="K9" s="0">
-        <v>3800</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="10">
@@ -551,28 +551,28 @@
         <v>8</v>
       </c>
       <c r="D10" s="0">
-        <v>0.82577077494129236</v>
+        <v>0.80683281569578058</v>
       </c>
       <c r="E10" s="0">
-        <v>0.708860759493671</v>
+        <v>0.73575129533678763</v>
       </c>
       <c r="F10" s="0">
-        <v>0.7466666666666667</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="G10" s="0">
-        <v>0.67469879518072284</v>
+        <v>0.85542168674698793</v>
       </c>
       <c r="H10" s="0">
-        <v>2800</v>
+        <v>3550</v>
       </c>
       <c r="I10" s="0">
-        <v>8101</v>
+        <v>7101</v>
       </c>
       <c r="J10" s="0">
-        <v>950</v>
+        <v>1950</v>
       </c>
       <c r="K10" s="0">
-        <v>1350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="11">
@@ -586,28 +586,28 @@
         <v>9</v>
       </c>
       <c r="D11" s="0">
-        <v>0.9090977956215438</v>
+        <v>0.88258465267782749</v>
       </c>
       <c r="E11" s="0">
-        <v>0.84615384615384603</v>
+        <v>0.82285714285714295</v>
       </c>
       <c r="F11" s="0">
-        <v>0.90410958904109584</v>
+        <v>0.78260869565217395</v>
       </c>
       <c r="G11" s="0">
-        <v>0.79518072289156627</v>
+        <v>0.86746987951807231</v>
       </c>
       <c r="H11" s="0">
-        <v>3300</v>
+        <v>3600</v>
       </c>
       <c r="I11" s="0">
-        <v>8701</v>
+        <v>8051</v>
       </c>
       <c r="J11" s="0">
-        <v>350</v>
+        <v>1000</v>
       </c>
       <c r="K11" s="0">
-        <v>850</v>
+        <v>550</v>
       </c>
     </row>
     <row r="12">
@@ -621,28 +621,28 @@
         <v>8</v>
       </c>
       <c r="D12" s="0">
-        <v>0.5808504191495808</v>
+        <v>0.60607005508782874</v>
       </c>
       <c r="E12" s="0">
-        <v>0.27826086956521745</v>
+        <v>0.44671532846715328</v>
       </c>
       <c r="F12" s="0">
-        <v>0.5</v>
+        <v>0.56666666666666665</v>
       </c>
       <c r="G12" s="0">
-        <v>0.19277108433734941</v>
+        <v>0.36867469879518072</v>
       </c>
       <c r="H12" s="0">
-        <v>800</v>
+        <v>1530</v>
       </c>
       <c r="I12" s="0">
-        <v>4951</v>
+        <v>4301</v>
       </c>
       <c r="J12" s="0">
-        <v>800</v>
+        <v>1170</v>
       </c>
       <c r="K12" s="0">
-        <v>3350</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="13">
@@ -656,28 +656,28 @@
         <v>9</v>
       </c>
       <c r="D13" s="0">
-        <v>0.78790021209978789</v>
+        <v>0.73831585378271047</v>
       </c>
       <c r="E13" s="0">
-        <v>0.73749999999999993</v>
+        <v>0.70289017341040461</v>
       </c>
       <c r="F13" s="0">
-        <v>0.76623376623376627</v>
+        <v>0.67555555555555558</v>
       </c>
       <c r="G13" s="0">
-        <v>0.71084337349397586</v>
+        <v>0.73253012048192767</v>
       </c>
       <c r="H13" s="0">
-        <v>2950</v>
+        <v>3040</v>
       </c>
       <c r="I13" s="0">
-        <v>4851</v>
+        <v>4211</v>
       </c>
       <c r="J13" s="0">
-        <v>900</v>
+        <v>1460</v>
       </c>
       <c r="K13" s="0">
-        <v>1200</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="14">
@@ -691,28 +691,28 @@
         <v>8</v>
       </c>
       <c r="D14" s="0">
-        <v>0.78023588015529999</v>
+        <v>0.81661761376499886</v>
       </c>
       <c r="E14" s="0">
-        <v>0.62500000000000011</v>
+        <v>0.75279755849440488</v>
       </c>
       <c r="F14" s="0">
-        <v>0.64935064935064934</v>
+        <v>0.61157024793388426</v>
       </c>
       <c r="G14" s="0">
-        <v>0.60240963855421692</v>
+        <v>0.97883597883597884</v>
       </c>
       <c r="H14" s="0">
-        <v>2500</v>
+        <v>3700</v>
       </c>
       <c r="I14" s="0">
-        <v>8151</v>
+        <v>7121</v>
       </c>
       <c r="J14" s="0">
-        <v>1350</v>
+        <v>2350</v>
       </c>
       <c r="K14" s="0">
-        <v>1650</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15">
@@ -726,28 +726,28 @@
         <v>9</v>
       </c>
       <c r="D15" s="0">
-        <v>0.87180426342392503</v>
+        <v>0.91753184596126947</v>
       </c>
       <c r="E15" s="0">
-        <v>0.7712418300653594</v>
+        <v>0.8752783964365255</v>
       </c>
       <c r="F15" s="0">
-        <v>0.84285714285714286</v>
+        <v>0.80204081632653057</v>
       </c>
       <c r="G15" s="0">
-        <v>0.71084337349397586</v>
+        <v>0.96323529411764708</v>
       </c>
       <c r="H15" s="0">
-        <v>2950</v>
+        <v>3930</v>
       </c>
       <c r="I15" s="0">
-        <v>8951</v>
+        <v>8531</v>
       </c>
       <c r="J15" s="0">
-        <v>550</v>
+        <v>970</v>
       </c>
       <c r="K15" s="0">
-        <v>1200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16">
@@ -761,28 +761,28 @@
         <v>8</v>
       </c>
       <c r="D16" s="0">
-        <v>0.75231630125676541</v>
+        <v>0.7110356847995597</v>
       </c>
       <c r="E16" s="0">
-        <v>0.7065217391304347</v>
+        <v>0.7069767441860465</v>
       </c>
       <c r="F16" s="0">
-        <v>0.64356435643564358</v>
+        <v>0.5757575757575758</v>
       </c>
       <c r="G16" s="0">
-        <v>0.7831325301204819</v>
+        <v>0.91566265060240959</v>
       </c>
       <c r="H16" s="0">
-        <v>3250</v>
+        <v>3800</v>
       </c>
       <c r="I16" s="0">
-        <v>4951</v>
+        <v>3951</v>
       </c>
       <c r="J16" s="0">
-        <v>1800</v>
+        <v>2800</v>
       </c>
       <c r="K16" s="0">
-        <v>900</v>
+        <v>350</v>
       </c>
     </row>
     <row r="17">
@@ -796,28 +796,28 @@
         <v>9</v>
       </c>
       <c r="D17" s="0">
-        <v>0.85140264790297193</v>
+        <v>0.73057118907915219</v>
       </c>
       <c r="E17" s="0">
-        <v>0.7841291190316072</v>
+        <v>0.73867595818815335</v>
       </c>
       <c r="F17" s="0">
-        <v>0.85735294117647054</v>
+        <v>0.594392523364486</v>
       </c>
       <c r="G17" s="0">
-        <v>0.72242874845105332</v>
+        <v>0.97546012269938653</v>
       </c>
       <c r="H17" s="0">
-        <v>2915</v>
+        <v>3180</v>
       </c>
       <c r="I17" s="0">
-        <v>6281</v>
+        <v>2921</v>
       </c>
       <c r="J17" s="0">
-        <v>485</v>
+        <v>2170</v>
       </c>
       <c r="K17" s="0">
-        <v>1120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18">
@@ -3353,7 +3353,7 @@
     <col min="2" max="2" width="10.88671875" customWidth="true"/>
     <col min="3" max="3" width="13.88671875" customWidth="true"/>
     <col min="4" max="4" width="13.88671875" customWidth="true"/>
-    <col min="5" max="5" width="11.5546875" customWidth="true"/>
+    <col min="5" max="5" width="12.5546875" customWidth="true"/>
     <col min="6" max="6" width="12.5546875" customWidth="true"/>
   </cols>
   <sheetData>
@@ -3385,16 +3385,16 @@
         <v>8</v>
       </c>
       <c r="C2" s="0">
-        <v>0.8628186691189097</v>
+        <v>0.86285633796038019</v>
       </c>
       <c r="D2" s="0">
-        <v>0.88626402390431447</v>
+        <v>0.79393017191882764</v>
       </c>
       <c r="E2" s="0">
-        <v>0.75520517800038978</v>
+        <v>0.90889277458394302</v>
       </c>
       <c r="F2" s="0">
-        <v>0.8136431892026792</v>
+        <v>0.84229990954944001</v>
       </c>
     </row>
     <row r="3">
@@ -3405,16 +3405,16 @@
         <v>8</v>
       </c>
       <c r="C3" s="0">
-        <v>0.78609871070904369</v>
+        <v>0.81291881570756941</v>
       </c>
       <c r="D3" s="0">
-        <v>0.76422004231926133</v>
+        <v>0.72422937769050599</v>
       </c>
       <c r="E3" s="0">
-        <v>0.64528677151570457</v>
+        <v>0.84874892434471394</v>
       </c>
       <c r="F3" s="0">
-        <v>0.6884624016777845</v>
+        <v>0.76989505398523628</v>
       </c>
     </row>
   </sheetData>
@@ -3462,16 +3462,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="0">
-        <v>0.833488390638083</v>
+        <v>0.95808309333956032</v>
       </c>
       <c r="D2" s="0">
-        <v>0.9600721247563353</v>
+        <v>0.92195428174014893</v>
       </c>
       <c r="E2" s="0">
-        <v>0.66633176458086796</v>
+        <v>0.97222150869658819</v>
       </c>
       <c r="F2" s="0">
-        <v>0.78586370485755297</v>
+        <v>0.94629221459311785</v>
       </c>
     </row>
     <row r="3">
@@ -3482,16 +3482,16 @@
         <v>2</v>
       </c>
       <c r="C3" s="0">
-        <v>0.91414504619129278</v>
+        <v>0.91771431682871829</v>
       </c>
       <c r="D3" s="0">
-        <v>0.97994124286283357</v>
+        <v>0.92348597622431294</v>
       </c>
       <c r="E3" s="0">
-        <v>0.83130656672381487</v>
+        <v>0.8966947091423787</v>
       </c>
       <c r="F3" s="0">
-        <v>0.89914734476009639</v>
+        <v>0.90985865929759058</v>
       </c>
     </row>
     <row r="4">
@@ -3502,16 +3502,16 @@
         <v>2</v>
       </c>
       <c r="C4" s="0">
-        <v>0.84644793331453105</v>
+        <v>0.83507248948955692</v>
       </c>
       <c r="D4" s="0">
-        <v>0.80633471143216262</v>
+        <v>0.72501385289123244</v>
       </c>
       <c r="E4" s="0">
-        <v>0.810546875</v>
+        <v>0.94832737862176975</v>
       </c>
       <c r="F4" s="0">
-        <v>0.8083867559936615</v>
+        <v>0.82176817785126999</v>
       </c>
     </row>
     <row r="5">
@@ -3522,16 +3522,16 @@
         <v>2</v>
       </c>
       <c r="C5" s="0">
-        <v>0.82189900189232312</v>
+        <v>0.88745085958939929</v>
       </c>
       <c r="D5" s="0">
-        <v>0.90052062996225435</v>
+        <v>0.87516077422593086</v>
       </c>
       <c r="E5" s="0">
-        <v>0.69762845849802368</v>
+        <v>0.88467798335509618</v>
       </c>
       <c r="F5" s="0">
-        <v>0.78619047619047622</v>
+        <v>0.87988950370841756</v>
       </c>
     </row>
     <row r="6">
@@ -3542,16 +3542,16 @@
         <v>2</v>
       </c>
       <c r="C6" s="0">
-        <v>0.86743428528141808</v>
+        <v>0.84470873418680403</v>
       </c>
       <c r="D6" s="0">
-        <v>0.82538812785388127</v>
+        <v>0.71403162055335967</v>
       </c>
       <c r="E6" s="0">
-        <v>0.73493975903614461</v>
+        <v>0.86144578313253017</v>
       </c>
       <c r="F6" s="0">
-        <v>0.77750730282375846</v>
+        <v>0.77930421909696523</v>
       </c>
     </row>
     <row r="7">
@@ -3562,16 +3562,16 @@
         <v>2</v>
       </c>
       <c r="C7" s="0">
-        <v>0.68437531562468434</v>
+        <v>0.67219295443526961</v>
       </c>
       <c r="D7" s="0">
-        <v>0.63311688311688319</v>
+        <v>0.62111111111111117</v>
       </c>
       <c r="E7" s="0">
-        <v>0.45180722891566261</v>
+        <v>0.55060240963855422</v>
       </c>
       <c r="F7" s="0">
-        <v>0.50788043478260869</v>
+        <v>0.57480275093877897</v>
       </c>
     </row>
     <row r="8">
@@ -3582,16 +3582,16 @@
         <v>2</v>
       </c>
       <c r="C8" s="0">
-        <v>0.82602007178961245</v>
+        <v>0.86707472986313416</v>
       </c>
       <c r="D8" s="0">
-        <v>0.74610389610389616</v>
+        <v>0.70680553213020736</v>
       </c>
       <c r="E8" s="0">
-        <v>0.65662650602409633</v>
+        <v>0.9710356364768129</v>
       </c>
       <c r="F8" s="0">
-        <v>0.6981209150326797</v>
+        <v>0.81403797746546513</v>
       </c>
     </row>
     <row r="9">
@@ -3602,16 +3602,16 @@
         <v>2</v>
       </c>
       <c r="C9" s="0">
-        <v>0.80185947457986861</v>
+        <v>0.72080343693935589</v>
       </c>
       <c r="D9" s="0">
-        <v>0.75045864880605706</v>
+        <v>0.58507504956103085</v>
       </c>
       <c r="E9" s="0">
-        <v>0.75278063928576766</v>
+        <v>0.94556138665089806</v>
       </c>
       <c r="F9" s="0">
-        <v>0.74532542908102095</v>
+        <v>0.72282635118709992</v>
       </c>
     </row>
     <row r="10">
@@ -3679,16 +3679,16 @@
         <v>6</v>
       </c>
       <c r="C2" s="0">
-        <v>0.82477582656133741</v>
+        <v>0.80765021876401555</v>
       </c>
       <c r="D2" s="0">
-        <v>0.76763241878070521</v>
+        <v>0.67229814486082373</v>
       </c>
       <c r="E2" s="0">
-        <v>0.73998467343662133</v>
+        <v>0.95497480058316031</v>
       </c>
       <c r="F2" s="0">
-        <v>0.75061103336912061</v>
+        <v>0.78621083550127846</v>
       </c>
     </row>
     <row r="3">
@@ -3699,16 +3699,16 @@
         <v>10</v>
       </c>
       <c r="C3" s="0">
-        <v>0.82426840792556022</v>
+        <v>0.85602999167595029</v>
       </c>
       <c r="D3" s="0">
-        <v>0.85980780171043758</v>
+        <v>0.81114875277097265</v>
       </c>
       <c r="E3" s="0">
-        <v>0.67640275555090279</v>
+        <v>0.83312847879302954</v>
       </c>
       <c r="F3" s="0">
-        <v>0.75131785268289852</v>
+        <v>0.81802946952697408</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Added freeliving scripts with plots
</commit_message>
<xml_diff>
--- a/mstraczkiewicz/MStraPlots_RT/Detailed_MStra_RT_Results.xlsx
+++ b/mstraczkiewicz/MStraPlots_RT/Detailed_MStra_RT_Results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3169" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3272" uniqueCount="51">
   <si>
     <t>Subject</t>
   </si>
@@ -164,6 +164,12 @@
   </si>
   <si>
     <t>test9</t>
+  </si>
+  <si>
+    <t>test10</t>
+  </si>
+  <si>
+    <t>test11</t>
   </si>
 </sst>
 </file>
@@ -262,212 +268,212 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="0">
-        <v>0.95912841879995459</v>
+        <v>0.75926146989773591</v>
       </c>
       <c r="E2" s="0">
-        <v>0.94395411395922724</v>
+        <v>0.71925754060324831</v>
       </c>
       <c r="F2" s="0">
-        <v>0.90920770877944324</v>
+        <v>0.82887700534759357</v>
       </c>
       <c r="G2" s="0">
-        <v>0.9814617909481762</v>
+        <v>0.63524590163934425</v>
       </c>
       <c r="H2" s="0">
-        <v>21230</v>
+        <v>7750</v>
       </c>
       <c r="I2" s="0">
-        <v>37930</v>
+        <v>11331</v>
       </c>
       <c r="J2" s="0">
-        <v>2120</v>
+        <v>1600</v>
       </c>
       <c r="K2" s="0">
-        <v>401</v>
+        <v>4450</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="0">
-        <v>0.95703776787916606</v>
+        <v>0.80900083562134417</v>
       </c>
       <c r="E3" s="0">
-        <v>0.94863031522700847</v>
+        <v>0.80165289256198347</v>
       </c>
       <c r="F3" s="0">
-        <v>0.93470085470085473</v>
+        <v>0.80833333333333335</v>
       </c>
       <c r="G3" s="0">
-        <v>0.96298122644500017</v>
+        <v>0.79508196721311475</v>
       </c>
       <c r="H3" s="0">
-        <v>27340</v>
+        <v>9700</v>
       </c>
       <c r="I3" s="0">
-        <v>38620</v>
+        <v>10631</v>
       </c>
       <c r="J3" s="0">
-        <v>1910</v>
+        <v>2300</v>
       </c>
       <c r="K3" s="0">
-        <v>1051</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="0">
-        <v>0.93153530819313313</v>
+        <v>0.93687107241138534</v>
       </c>
       <c r="E4" s="0">
-        <v>0.92578070016689784</v>
+        <v>0.93963948632692329</v>
       </c>
       <c r="F4" s="0">
-        <v>0.93387423935091274</v>
+        <v>0.98194254445964435</v>
       </c>
       <c r="G4" s="0">
-        <v>0.91782624297276827</v>
+        <v>0.90083080243969782</v>
       </c>
       <c r="H4" s="0">
-        <v>23020</v>
+        <v>35890</v>
       </c>
       <c r="I4" s="0">
-        <v>27200</v>
+        <v>32540</v>
       </c>
       <c r="J4" s="0">
-        <v>1630</v>
+        <v>660</v>
       </c>
       <c r="K4" s="0">
-        <v>2061</v>
+        <v>3951</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="0">
-        <v>0.90389332546430345</v>
+        <v>0.95565738839558889</v>
       </c>
       <c r="E5" s="0">
-        <v>0.89393661842828342</v>
+        <v>0.95900227555600259</v>
       </c>
       <c r="F5" s="0">
-        <v>0.91309771309771315</v>
+        <v>0.97295918367346934</v>
       </c>
       <c r="G5" s="0">
-        <v>0.87556317531198913</v>
+        <v>0.94544012295183555</v>
       </c>
       <c r="H5" s="0">
-        <v>21960</v>
+        <v>38140</v>
       </c>
       <c r="I5" s="0">
-        <v>27050</v>
+        <v>32140</v>
       </c>
       <c r="J5" s="0">
-        <v>2090</v>
+        <v>1060</v>
       </c>
       <c r="K5" s="0">
-        <v>3121</v>
+        <v>2201</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="0">
-        <v>0.79988080675010198</v>
+        <v>0.8316985781683176</v>
       </c>
       <c r="E6" s="0">
-        <v>0.78387533875338755</v>
+        <v>0.7065939345976654</v>
       </c>
       <c r="F6" s="0">
-        <v>0.6907462686567164</v>
+        <v>0.90909090909090906</v>
       </c>
       <c r="G6" s="0">
-        <v>0.90602975724353951</v>
+        <v>0.57787434700198792</v>
       </c>
       <c r="H6" s="0">
-        <v>11570</v>
+        <v>12500</v>
       </c>
       <c r="I6" s="0">
-        <v>13931</v>
+        <v>38800</v>
       </c>
       <c r="J6" s="0">
-        <v>5180</v>
+        <v>1250</v>
       </c>
       <c r="K6" s="0">
-        <v>1200</v>
+        <v>9131</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="0">
-        <v>0.87026417222901198</v>
+        <v>0.9341129699220847</v>
       </c>
       <c r="E7" s="0">
-        <v>0.85966101694915253</v>
+        <v>0.91794510399161555</v>
       </c>
       <c r="F7" s="0">
-        <v>0.75928143712574847</v>
+        <v>0.9424860853432282</v>
       </c>
       <c r="G7" s="0">
-        <v>0.99062499999999998</v>
+        <v>0.89464971293719842</v>
       </c>
       <c r="H7" s="0">
-        <v>12680</v>
+        <v>25400</v>
       </c>
       <c r="I7" s="0">
-        <v>15091</v>
+        <v>38980</v>
       </c>
       <c r="J7" s="0">
-        <v>4020</v>
+        <v>1550</v>
       </c>
       <c r="K7" s="0">
-        <v>120</v>
+        <v>2991</v>
       </c>
     </row>
     <row r="8">
@@ -475,34 +481,34 @@
         <v>1</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="0">
-        <v>0.87224982256919803</v>
+        <v>0.93431767171820224</v>
       </c>
       <c r="E8" s="0">
-        <v>0.86330935251798557</v>
+        <v>0.92726114911361723</v>
       </c>
       <c r="F8" s="0">
-        <v>0.8605577689243028</v>
+        <v>0.95635593220338988</v>
       </c>
       <c r="G8" s="0">
-        <v>0.8660785886126704</v>
+        <v>0.89988437462621107</v>
       </c>
       <c r="H8" s="0">
-        <v>10800</v>
+        <v>22570</v>
       </c>
       <c r="I8" s="0">
-        <v>12551</v>
+        <v>27800</v>
       </c>
       <c r="J8" s="0">
-        <v>1750</v>
+        <v>1030</v>
       </c>
       <c r="K8" s="0">
-        <v>1670</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="9">
@@ -510,104 +516,104 @@
         <v>1</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="0">
-        <v>0.90265189660960055</v>
+        <v>0.90112686966304567</v>
       </c>
       <c r="E9" s="0">
-        <v>0.89646965489884956</v>
+        <v>0.88709167877677386</v>
       </c>
       <c r="F9" s="0">
-        <v>0.88976377952755903</v>
+        <v>0.94017857142857142</v>
       </c>
       <c r="G9" s="0">
-        <v>0.90327737809752195</v>
+        <v>0.83967943861887484</v>
       </c>
       <c r="H9" s="0">
-        <v>11300</v>
+        <v>21060</v>
       </c>
       <c r="I9" s="0">
-        <v>12901</v>
+        <v>27800</v>
       </c>
       <c r="J9" s="0">
-        <v>1400</v>
+        <v>1340</v>
       </c>
       <c r="K9" s="0">
-        <v>1210</v>
+        <v>4021</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="0">
-        <v>0.80683281569578058</v>
+        <v>0.78921614754869673</v>
       </c>
       <c r="E10" s="0">
-        <v>0.73575129533678763</v>
+        <v>0.75129533678756477</v>
       </c>
       <c r="F10" s="0">
-        <v>0.6454545454545455</v>
+        <v>0.71228070175438596</v>
       </c>
       <c r="G10" s="0">
-        <v>0.85542168674698793</v>
+        <v>0.79483163664839462</v>
       </c>
       <c r="H10" s="0">
-        <v>3550</v>
+        <v>10150</v>
       </c>
       <c r="I10" s="0">
-        <v>7101</v>
+        <v>15011</v>
       </c>
       <c r="J10" s="0">
-        <v>1950</v>
+        <v>4100</v>
       </c>
       <c r="K10" s="0">
-        <v>600</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="0">
-        <v>0.88258465267782749</v>
+        <v>0.88123217699225975</v>
       </c>
       <c r="E11" s="0">
-        <v>0.82285714285714295</v>
+        <v>0.86243194192377493</v>
       </c>
       <c r="F11" s="0">
-        <v>0.78260869565217395</v>
+        <v>0.80542372881355928</v>
       </c>
       <c r="G11" s="0">
-        <v>0.86746987951807231</v>
+        <v>0.92812499999999998</v>
       </c>
       <c r="H11" s="0">
-        <v>3600</v>
+        <v>11880</v>
       </c>
       <c r="I11" s="0">
-        <v>8051</v>
+        <v>16241</v>
       </c>
       <c r="J11" s="0">
-        <v>1000</v>
+        <v>2870</v>
       </c>
       <c r="K11" s="0">
-        <v>550</v>
+        <v>920</v>
       </c>
     </row>
     <row r="12">
@@ -615,34 +621,34 @@
         <v>1</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="0">
-        <v>0.60607005508782874</v>
+        <v>0.85992305106271716</v>
       </c>
       <c r="E12" s="0">
-        <v>0.44671532846715328</v>
+        <v>0.84289903644742348</v>
       </c>
       <c r="F12" s="0">
-        <v>0.56666666666666665</v>
+        <v>0.88245614035087716</v>
       </c>
       <c r="G12" s="0">
-        <v>0.36867469879518072</v>
+        <v>0.80673616680032079</v>
       </c>
       <c r="H12" s="0">
-        <v>1530</v>
+        <v>10060</v>
       </c>
       <c r="I12" s="0">
-        <v>4301</v>
+        <v>12961</v>
       </c>
       <c r="J12" s="0">
-        <v>1170</v>
+        <v>1340</v>
       </c>
       <c r="K12" s="0">
-        <v>2620</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="13">
@@ -650,314 +656,314 @@
         <v>1</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="0">
-        <v>0.73831585378271047</v>
+        <v>0.87094849129088803</v>
       </c>
       <c r="E13" s="0">
-        <v>0.70289017341040461</v>
+        <v>0.85619285120532007</v>
       </c>
       <c r="F13" s="0">
-        <v>0.67555555555555558</v>
+        <v>0.89177489177489178</v>
       </c>
       <c r="G13" s="0">
-        <v>0.73253012048192767</v>
+        <v>0.82334132693844919</v>
       </c>
       <c r="H13" s="0">
-        <v>3040</v>
+        <v>10300</v>
       </c>
       <c r="I13" s="0">
-        <v>4211</v>
+        <v>13051</v>
       </c>
       <c r="J13" s="0">
-        <v>1460</v>
+        <v>1250</v>
       </c>
       <c r="K13" s="0">
-        <v>1110</v>
+        <v>2210</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="0">
-        <v>0.81661761376499886</v>
+        <v>0.80304522384667831</v>
       </c>
       <c r="E14" s="0">
-        <v>0.75279755849440488</v>
+        <v>0.7078651685393258</v>
       </c>
       <c r="F14" s="0">
-        <v>0.61157024793388426</v>
+        <v>0.66315789473684206</v>
       </c>
       <c r="G14" s="0">
-        <v>0.97883597883597884</v>
+        <v>0.75903614457831325</v>
       </c>
       <c r="H14" s="0">
-        <v>3700</v>
+        <v>3150</v>
       </c>
       <c r="I14" s="0">
-        <v>7121</v>
+        <v>7451</v>
       </c>
       <c r="J14" s="0">
-        <v>2350</v>
+        <v>1600</v>
       </c>
       <c r="K14" s="0">
-        <v>80</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="0">
-        <v>0.91753184596126947</v>
+        <v>0.88637224452692975</v>
       </c>
       <c r="E15" s="0">
-        <v>0.8752783964365255</v>
+        <v>0.82352941176470607</v>
       </c>
       <c r="F15" s="0">
-        <v>0.80204081632653057</v>
+        <v>0.8045977011494253</v>
       </c>
       <c r="G15" s="0">
-        <v>0.96323529411764708</v>
+        <v>0.84337349397590367</v>
       </c>
       <c r="H15" s="0">
-        <v>3930</v>
+        <v>3500</v>
       </c>
       <c r="I15" s="0">
-        <v>8531</v>
+        <v>8201</v>
       </c>
       <c r="J15" s="0">
-        <v>970</v>
+        <v>850</v>
       </c>
       <c r="K15" s="0">
-        <v>150</v>
+        <v>650</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="0">
-        <v>0.7110356847995597</v>
+        <v>0.55306101236877658</v>
       </c>
       <c r="E16" s="0">
-        <v>0.7069767441860465</v>
+        <v>0.28333333333333333</v>
       </c>
       <c r="F16" s="0">
-        <v>0.5757575757575758</v>
+        <v>0.45945945945945948</v>
       </c>
       <c r="G16" s="0">
-        <v>0.91566265060240959</v>
+        <v>0.20481927710843373</v>
       </c>
       <c r="H16" s="0">
-        <v>3800</v>
+        <v>850</v>
       </c>
       <c r="I16" s="0">
-        <v>3951</v>
+        <v>4471</v>
       </c>
       <c r="J16" s="0">
-        <v>2800</v>
+        <v>1000</v>
       </c>
       <c r="K16" s="0">
-        <v>350</v>
+        <v>3300</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C17" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="0">
-        <v>0.73057118907915219</v>
+        <v>0.70776906628652891</v>
       </c>
       <c r="E17" s="0">
-        <v>0.73867595818815335</v>
+        <v>0.65212121212121221</v>
       </c>
       <c r="F17" s="0">
-        <v>0.594392523364486</v>
+        <v>0.65609756097560978</v>
       </c>
       <c r="G17" s="0">
-        <v>0.97546012269938653</v>
+        <v>0.64819277108433737</v>
       </c>
       <c r="H17" s="0">
-        <v>3180</v>
+        <v>2690</v>
       </c>
       <c r="I17" s="0">
-        <v>2921</v>
+        <v>4261</v>
       </c>
       <c r="J17" s="0">
-        <v>2170</v>
+        <v>1410</v>
       </c>
       <c r="K17" s="0">
-        <v>80</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C18" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="0">
-        <v>0.91922666350373616</v>
+        <v>0.79775111312353786</v>
       </c>
       <c r="E18" s="0">
-        <v>0.95791360237315371</v>
+        <v>0.6912442396313363</v>
       </c>
       <c r="F18" s="0">
-        <v>1</v>
+        <v>0.61224489795918369</v>
       </c>
       <c r="G18" s="0">
-        <v>0.91922666350373616</v>
+        <v>0.79365079365079361</v>
       </c>
       <c r="H18" s="0">
-        <v>7750</v>
+        <v>3000</v>
       </c>
       <c r="I18" s="0">
-        <v>0</v>
+        <v>7571</v>
       </c>
       <c r="J18" s="0">
-        <v>0</v>
+        <v>1900</v>
       </c>
       <c r="K18" s="0">
-        <v>681</v>
+        <v>780</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C19" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D19" s="0">
-        <v>0.40327363302099395</v>
+        <v>0.89617848464766958</v>
       </c>
       <c r="E19" s="0">
-        <v>0.57476122052235656</v>
+        <v>0.82656826568265673</v>
       </c>
       <c r="F19" s="0">
-        <v>1</v>
+        <v>0.82962962962962961</v>
       </c>
       <c r="G19" s="0">
-        <v>0.40327363302099395</v>
+        <v>0.82352941176470584</v>
       </c>
       <c r="H19" s="0">
-        <v>3400</v>
+        <v>3360</v>
       </c>
       <c r="I19" s="0">
-        <v>0</v>
+        <v>8811</v>
       </c>
       <c r="J19" s="0">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="K19" s="0">
-        <v>5031</v>
+        <v>720</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C20" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="0">
-        <v>0.71755243652420753</v>
+        <v>0.71562241996147147</v>
       </c>
       <c r="E20" s="0">
-        <v>0.83555229088238003</v>
+        <v>0.68686868686868674</v>
       </c>
       <c r="F20" s="0">
-        <v>1</v>
+        <v>0.59130434782608698</v>
       </c>
       <c r="G20" s="0">
-        <v>0.71755243652420753</v>
+        <v>0.81927710843373491</v>
       </c>
       <c r="H20" s="0">
-        <v>4550</v>
+        <v>3400</v>
       </c>
       <c r="I20" s="0">
-        <v>0</v>
+        <v>4401</v>
       </c>
       <c r="J20" s="0">
-        <v>0</v>
+        <v>2350</v>
       </c>
       <c r="K20" s="0">
-        <v>1791</v>
+        <v>750</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C21" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D21" s="0">
-        <v>0.96199337643904748</v>
+        <v>0.81199856304634177</v>
       </c>
       <c r="E21" s="0">
-        <v>0.98062856683546329</v>
+        <v>0.70979667282809611</v>
       </c>
       <c r="F21" s="0">
-        <v>1</v>
+        <v>0.89302325581395348</v>
       </c>
       <c r="G21" s="0">
-        <v>0.96199337643904748</v>
+        <v>0.58895705521472397</v>
       </c>
       <c r="H21" s="0">
-        <v>6100</v>
+        <v>1920</v>
       </c>
       <c r="I21" s="0">
-        <v>0</v>
+        <v>4861</v>
       </c>
       <c r="J21" s="0">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="K21" s="0">
-        <v>241</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="22">
@@ -3382,19 +3388,19 @@
         <v>9</v>
       </c>
       <c r="B2" s="0">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" s="0">
-        <v>0.86285633796038019</v>
+        <v>0.86543970903926815</v>
       </c>
       <c r="D2" s="0">
-        <v>0.79393017191882764</v>
+        <v>0.85445039419356728</v>
       </c>
       <c r="E2" s="0">
-        <v>0.90889277458394302</v>
+        <v>0.81303703006991435</v>
       </c>
       <c r="F2" s="0">
-        <v>0.84229990954944001</v>
+        <v>0.82963323064121419</v>
       </c>
     </row>
     <row r="3">
@@ -3402,19 +3408,19 @@
         <v>8</v>
       </c>
       <c r="B3" s="0">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C3" s="0">
-        <v>0.81291881570756941</v>
+        <v>0.79807677601075189</v>
       </c>
       <c r="D3" s="0">
-        <v>0.72422937769050599</v>
+        <v>0.7597169833188373</v>
       </c>
       <c r="E3" s="0">
-        <v>0.84874892434471394</v>
+        <v>0.71921865529272322</v>
       </c>
       <c r="F3" s="0">
-        <v>0.76989505398523628</v>
+        <v>0.72562579122491244</v>
       </c>
     </row>
   </sheetData>
@@ -3423,7 +3429,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="true"/>
@@ -3462,176 +3468,196 @@
         <v>2</v>
       </c>
       <c r="C2" s="0">
-        <v>0.95808309333956032</v>
+        <v>0.8829057740452011</v>
       </c>
       <c r="D2" s="0">
-        <v>0.92195428174014893</v>
+        <v>0.92578849721706868</v>
       </c>
       <c r="E2" s="0">
-        <v>0.97222150869658819</v>
+        <v>0.73626202996959322</v>
       </c>
       <c r="F2" s="0">
-        <v>0.94629221459311785</v>
+        <v>0.81226951929464053</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="B3" s="0">
         <v>2</v>
       </c>
       <c r="C3" s="0">
-        <v>0.91771431682871829</v>
+        <v>0.78413115275954004</v>
       </c>
       <c r="D3" s="0">
-        <v>0.92348597622431294</v>
+        <v>0.81860516934046346</v>
       </c>
       <c r="E3" s="0">
-        <v>0.8966947091423787</v>
+        <v>0.7151639344262295</v>
       </c>
       <c r="F3" s="0">
-        <v>0.90985865929759058</v>
+        <v>0.76045521658261594</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="B4" s="0">
         <v>2</v>
       </c>
       <c r="C4" s="0">
-        <v>0.83507248948955692</v>
+        <v>0.94626423040348717</v>
       </c>
       <c r="D4" s="0">
-        <v>0.72501385289123244</v>
+        <v>0.9774508640665569</v>
       </c>
       <c r="E4" s="0">
-        <v>0.94832737862176975</v>
+        <v>0.92313546269576663</v>
       </c>
       <c r="F4" s="0">
-        <v>0.82176817785126999</v>
+        <v>0.94932088094146294</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="B5" s="0">
         <v>2</v>
       </c>
       <c r="C5" s="0">
-        <v>0.88745085958939929</v>
+        <v>0.91772227069062395</v>
       </c>
       <c r="D5" s="0">
-        <v>0.87516077422593086</v>
+        <v>0.94826725181598071</v>
       </c>
       <c r="E5" s="0">
-        <v>0.88467798335509618</v>
+        <v>0.86978190662254296</v>
       </c>
       <c r="F5" s="0">
-        <v>0.87988950370841756</v>
+        <v>0.90717641394519555</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="B6" s="0">
         <v>2</v>
       </c>
       <c r="C6" s="0">
-        <v>0.84470873418680403</v>
+        <v>0.83522416227047824</v>
       </c>
       <c r="D6" s="0">
-        <v>0.71403162055335967</v>
+        <v>0.75885221528397262</v>
       </c>
       <c r="E6" s="0">
-        <v>0.86144578313253017</v>
+        <v>0.8614783183241973</v>
       </c>
       <c r="F6" s="0">
-        <v>0.77930421909696523</v>
+        <v>0.80686363935566985</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B7" s="0">
         <v>2</v>
       </c>
       <c r="C7" s="0">
-        <v>0.67219295443526961</v>
+        <v>0.86543577117680259</v>
       </c>
       <c r="D7" s="0">
-        <v>0.62111111111111117</v>
+        <v>0.88711551606288452</v>
       </c>
       <c r="E7" s="0">
-        <v>0.55060240963855422</v>
+        <v>0.81503874686938493</v>
       </c>
       <c r="F7" s="0">
-        <v>0.57480275093877897</v>
+        <v>0.84954594382637172</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B8" s="0">
         <v>2</v>
       </c>
       <c r="C8" s="0">
-        <v>0.86707472986313416</v>
+        <v>0.84470873418680403</v>
       </c>
       <c r="D8" s="0">
-        <v>0.70680553213020736</v>
+        <v>0.73387779794313368</v>
       </c>
       <c r="E8" s="0">
-        <v>0.9710356364768129</v>
+        <v>0.8012048192771084</v>
       </c>
       <c r="F8" s="0">
-        <v>0.81403797746546513</v>
+        <v>0.76569729015201593</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="0">
         <v>2</v>
       </c>
       <c r="C9" s="0">
-        <v>0.72080343693935589</v>
+        <v>0.63041503932765275</v>
       </c>
       <c r="D9" s="0">
-        <v>0.58507504956103085</v>
+        <v>0.55777851021753466</v>
       </c>
       <c r="E9" s="0">
-        <v>0.94556138665089806</v>
+        <v>0.42650602409638555</v>
       </c>
       <c r="F9" s="0">
-        <v>0.72282635118709992</v>
+        <v>0.46772727272727277</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="B10" s="0">
         <v>2</v>
       </c>
       <c r="C10" s="0">
-        <v>0.84629124753219898</v>
+        <v>0.84696479888560372</v>
       </c>
       <c r="D10" s="0">
-        <v>0.80593945451516658</v>
+        <v>0.7209372637944067</v>
       </c>
       <c r="E10" s="0">
-        <v>0.81044120162236122</v>
+        <v>0.80859010270774978</v>
       </c>
       <c r="F10" s="0">
-        <v>0.80813793292215608</v>
+        <v>0.75890625265699652</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="0">
+        <v>2</v>
+      </c>
+      <c r="C11" s="0">
+        <v>0.76381049150390656</v>
+      </c>
+      <c r="D11" s="0">
+        <v>0.74216380182002029</v>
+      </c>
+      <c r="E11" s="0">
+        <v>0.7041170818242295</v>
+      </c>
+      <c r="F11" s="0">
+        <v>0.69833267984839142</v>
       </c>
     </row>
   </sheetData>
@@ -3647,7 +3673,7 @@
     <col min="2" max="2" width="10.88671875" customWidth="true"/>
     <col min="3" max="3" width="13.88671875" customWidth="true"/>
     <col min="4" max="4" width="13.88671875" customWidth="true"/>
-    <col min="5" max="5" width="12.5546875" customWidth="true"/>
+    <col min="5" max="5" width="11.44140625" customWidth="true"/>
     <col min="6" max="6" width="12.5546875" customWidth="true"/>
   </cols>
   <sheetData>
@@ -3676,19 +3702,19 @@
         <v>2</v>
       </c>
       <c r="B2" s="0">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C2" s="0">
-        <v>0.80765021876401555</v>
+        <v>0.83527896716460304</v>
       </c>
       <c r="D2" s="0">
-        <v>0.67229814486082373</v>
+        <v>0.80360186286108404</v>
       </c>
       <c r="E2" s="0">
-        <v>0.95497480058316031</v>
+        <v>0.80249697999563452</v>
       </c>
       <c r="F2" s="0">
-        <v>0.78621083550127846</v>
+        <v>0.79477573387702738</v>
       </c>
     </row>
     <row r="3">
@@ -3699,16 +3725,16 @@
         <v>10</v>
       </c>
       <c r="C3" s="0">
-        <v>0.85602999167595029</v>
+        <v>0.82823751788541689</v>
       </c>
       <c r="D3" s="0">
-        <v>0.81114875277097265</v>
+        <v>0.81056551465132043</v>
       </c>
       <c r="E3" s="0">
-        <v>0.83312847879302954</v>
+        <v>0.72975870536700294</v>
       </c>
       <c r="F3" s="0">
-        <v>0.81802946952697408</v>
+        <v>0.76048328798909925</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Retrained ElderNet (strokenet) and processed on all datasets
</commit_message>
<xml_diff>
--- a/mstraczkiewicz/MStraPlots_RT/Detailed_MStra_RT_Results.xlsx
+++ b/mstraczkiewicz/MStraPlots_RT/Detailed_MStra_RT_Results.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="15572" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="15728" uniqueCount="67">
   <si>
     <t>Subject</t>
   </si>
@@ -217,6 +217,9 @@
   <si>
     <t>EvaluableSec</t>
   </si>
+  <si>
+    <t>Hub</t>
+  </si>
 </sst>
 </file>
 
@@ -264,17 +267,17 @@
   <dimension ref="A1:K105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" customWidth="true"/>
-    <col min="2" max="2" width="9.88671875" customWidth="true"/>
+    <col min="1" max="1" width="6.88671875" customWidth="true"/>
+    <col min="2" max="2" width="8.88671875" customWidth="true"/>
     <col min="3" max="3" width="5.33203125" customWidth="true"/>
     <col min="4" max="4" width="12.5546875" customWidth="true"/>
-    <col min="5" max="5" width="12.5546875" customWidth="true"/>
-    <col min="6" max="6" width="12.5546875" customWidth="true"/>
-    <col min="7" max="7" width="12.5546875" customWidth="true"/>
-    <col min="8" max="8" width="6" customWidth="true"/>
+    <col min="5" max="5" width="2.88671875" customWidth="true"/>
+    <col min="6" max="6" width="8.33203125" customWidth="true"/>
+    <col min="7" max="7" width="5.88671875" customWidth="true"/>
+    <col min="8" max="8" width="3" customWidth="true"/>
     <col min="9" max="9" width="8" customWidth="true"/>
     <col min="10" max="10" width="6" customWidth="true"/>
-    <col min="11" max="11" width="5" customWidth="true"/>
+    <col min="11" max="11" width="3.21875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -314,142 +317,142 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="0">
-        <v>0.83684838838042186</v>
+        <v>0.3602540834845735</v>
       </c>
       <c r="E2" s="0">
-        <v>0.8423076923076922</v>
+        <v>0</v>
       </c>
       <c r="F2" s="0">
-        <v>0.79347826086956519</v>
+        <v>0</v>
       </c>
       <c r="G2" s="0">
-        <v>0.89754098360655743</v>
+        <v>1</v>
       </c>
       <c r="H2" s="0">
-        <v>10950</v>
+        <v>0</v>
       </c>
       <c r="I2" s="0">
-        <v>10080</v>
+        <v>7940</v>
       </c>
       <c r="J2" s="0">
-        <v>2850</v>
+        <v>14100</v>
       </c>
       <c r="K2" s="0">
-        <v>1250</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="0">
-        <v>0.84480700358137684</v>
+        <v>0.3693101830126701</v>
       </c>
       <c r="E3" s="0">
-        <v>0.84999999999999998</v>
+        <v>0</v>
       </c>
       <c r="F3" s="0">
-        <v>0.80072463768115942</v>
+        <v>0</v>
       </c>
       <c r="G3" s="0">
-        <v>0.90573770491803274</v>
+        <v>1</v>
       </c>
       <c r="H3" s="0">
-        <v>11050</v>
+        <v>0</v>
       </c>
       <c r="I3" s="0">
-        <v>10180</v>
+        <v>7870</v>
       </c>
       <c r="J3" s="0">
-        <v>2750</v>
+        <v>13440</v>
       </c>
       <c r="K3" s="0">
-        <v>1150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="0">
-        <v>0.97598870056497178</v>
+        <v>0.98328781304376556</v>
       </c>
       <c r="E4" s="0">
-        <v>0.97735748534896105</v>
+        <v>0</v>
       </c>
       <c r="F4" s="0">
-        <v>0.97892209178228384</v>
+        <v>0</v>
       </c>
       <c r="G4" s="0">
-        <v>0.97579787234042559</v>
+        <v>1</v>
       </c>
       <c r="H4" s="0">
-        <v>36690</v>
+        <v>0</v>
       </c>
       <c r="I4" s="0">
-        <v>32410</v>
+        <v>1785690</v>
       </c>
       <c r="J4" s="0">
-        <v>790</v>
+        <v>30350</v>
       </c>
       <c r="K4" s="0">
-        <v>910</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="0">
-        <v>0.97780501089324623</v>
+        <v>0.98421887565685828</v>
       </c>
       <c r="E5" s="0">
-        <v>0.97991868917087588</v>
+        <v>0</v>
       </c>
       <c r="F5" s="0">
-        <v>0.97165892988028346</v>
+        <v>0</v>
       </c>
       <c r="G5" s="0">
-        <v>0.98832007952286283</v>
+        <v>1</v>
       </c>
       <c r="H5" s="0">
-        <v>39770</v>
+        <v>0</v>
       </c>
       <c r="I5" s="0">
-        <v>32040</v>
+        <v>1786810</v>
       </c>
       <c r="J5" s="0">
-        <v>1160</v>
+        <v>28650</v>
       </c>
       <c r="K5" s="0">
-        <v>470</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3967,10 +3970,10 @@
     <col min="4" max="4" width="7.21875" customWidth="true"/>
     <col min="5" max="5" width="8" customWidth="true"/>
     <col min="6" max="6" width="7.5546875" customWidth="true"/>
-    <col min="7" max="7" width="12.5546875" customWidth="true"/>
-    <col min="8" max="8" width="12.5546875" customWidth="true"/>
+    <col min="7" max="7" width="8.33203125" customWidth="true"/>
+    <col min="8" max="8" width="5.88671875" customWidth="true"/>
     <col min="9" max="9" width="12.5546875" customWidth="true"/>
-    <col min="10" max="10" width="12.5546875" customWidth="true"/>
+    <col min="10" max="10" width="2.88671875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4010,31 +4013,31 @@
         <v>9</v>
       </c>
       <c r="B2" s="0">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="C2" s="0">
-        <v>304870</v>
+        <v>0</v>
       </c>
       <c r="D2" s="0">
-        <v>71650</v>
+        <v>42090</v>
       </c>
       <c r="E2" s="0">
-        <v>2731720</v>
+        <v>1794680</v>
       </c>
       <c r="F2" s="0">
-        <v>36160</v>
+        <v>0</v>
       </c>
       <c r="G2" s="0">
-        <v>0.80970466376288108</v>
+        <v>0</v>
       </c>
       <c r="H2" s="0">
-        <v>0.89396827258598954</v>
+        <v>0</v>
       </c>
       <c r="I2" s="0">
-        <v>0.96571364966289275</v>
+        <v>0.97708477381490333</v>
       </c>
       <c r="J2" s="0">
-        <v>0.84975263047871241</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -4042,31 +4045,31 @@
         <v>8</v>
       </c>
       <c r="B3" s="0">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="C3" s="0">
-        <v>279590</v>
+        <v>0</v>
       </c>
       <c r="D3" s="0">
-        <v>107530</v>
+        <v>44450</v>
       </c>
       <c r="E3" s="0">
-        <v>2695670</v>
+        <v>1793630</v>
       </c>
       <c r="F3" s="0">
-        <v>43390</v>
+        <v>0</v>
       </c>
       <c r="G3" s="0">
-        <v>0.72223083281669764</v>
+        <v>0</v>
       </c>
       <c r="H3" s="0">
-        <v>0.86565731624249176</v>
+        <v>0</v>
       </c>
       <c r="I3" s="0">
-        <v>0.95172382908213859</v>
+        <v>0.9758171570334262</v>
       </c>
       <c r="J3" s="0">
-        <v>0.78746655400647791</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4078,16 +4081,16 @@
   <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" customWidth="true"/>
+    <col min="1" max="1" width="7" customWidth="true"/>
     <col min="2" max="2" width="10.88671875" customWidth="true"/>
     <col min="3" max="3" width="7.33203125" customWidth="true"/>
     <col min="4" max="4" width="7.21875" customWidth="true"/>
-    <col min="5" max="5" width="8" customWidth="true"/>
+    <col min="5" max="5" width="7.6640625" customWidth="true"/>
     <col min="6" max="6" width="7.5546875" customWidth="true"/>
-    <col min="7" max="7" width="12.5546875" customWidth="true"/>
-    <col min="8" max="8" width="12.5546875" customWidth="true"/>
+    <col min="7" max="7" width="8.33203125" customWidth="true"/>
+    <col min="8" max="8" width="5.88671875" customWidth="true"/>
     <col min="9" max="9" width="12.5546875" customWidth="true"/>
-    <col min="10" max="10" width="12.5546875" customWidth="true"/>
+    <col min="10" max="10" width="2.88671875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4124,19 +4127,19 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="B2" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C2" s="0">
         <v>0</v>
       </c>
       <c r="D2" s="0">
-        <v>65110</v>
+        <v>27540</v>
       </c>
       <c r="E2" s="0">
-        <v>1481180</v>
+        <v>15810</v>
       </c>
       <c r="F2" s="0">
         <v>0</v>
@@ -4148,7 +4151,7 @@
         <v>0</v>
       </c>
       <c r="I2" s="0">
-        <v>0.95789276267711754</v>
+        <v>0.36470588235294116</v>
       </c>
       <c r="J2" s="0">
         <v>0</v>
@@ -4156,19 +4159,19 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="B3" s="0">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3" s="0">
         <v>0</v>
       </c>
       <c r="D3" s="0">
-        <v>250</v>
+        <v>59000</v>
       </c>
       <c r="E3" s="0">
-        <v>30600</v>
+        <v>3572500</v>
       </c>
       <c r="F3" s="0">
         <v>0</v>
@@ -4180,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="0">
-        <v>0.99189627228525123</v>
+        <v>0.98375326999862311</v>
       </c>
       <c r="J3" s="0">
         <v>0</v>
@@ -4675,16 +4678,16 @@
   <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" customWidth="true"/>
+    <col min="1" max="1" width="6.88671875" customWidth="true"/>
     <col min="2" max="2" width="10.88671875" customWidth="true"/>
     <col min="3" max="3" width="7.33203125" customWidth="true"/>
     <col min="4" max="4" width="7.21875" customWidth="true"/>
-    <col min="5" max="5" width="8" customWidth="true"/>
+    <col min="5" max="5" width="7.6640625" customWidth="true"/>
     <col min="6" max="6" width="7.5546875" customWidth="true"/>
-    <col min="7" max="7" width="12.5546875" customWidth="true"/>
-    <col min="8" max="8" width="12.5546875" customWidth="true"/>
-    <col min="9" max="9" width="12.5546875" customWidth="true"/>
-    <col min="10" max="10" width="12.5546875" customWidth="true"/>
+    <col min="7" max="7" width="8.33203125" customWidth="true"/>
+    <col min="8" max="8" width="5.88671875" customWidth="true"/>
+    <col min="9" max="9" width="8.33203125" customWidth="true"/>
+    <col min="10" max="10" width="2.88671875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4721,34 +4724,34 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B2" s="0">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C2" s="0">
-        <v>154410</v>
+        <v>0</v>
       </c>
       <c r="D2" s="0">
-        <v>67290</v>
+        <v>86540</v>
       </c>
       <c r="E2" s="0">
-        <v>963850</v>
+        <v>3588310</v>
       </c>
       <c r="F2" s="0">
-        <v>5520</v>
+        <v>0</v>
       </c>
       <c r="G2" s="0">
-        <v>0.69648173207036534</v>
+        <v>0</v>
       </c>
       <c r="H2" s="0">
-        <v>0.96548489964359407</v>
+        <v>0</v>
       </c>
       <c r="I2" s="0">
-        <v>0.93887009159831081</v>
+        <v>0.97645073948596539</v>
       </c>
       <c r="J2" s="0">
-        <v>0.80921311217671565</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -5304,12 +5307,12 @@
   <dimension ref="A1:H105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" customWidth="true"/>
-    <col min="2" max="2" width="9.88671875" customWidth="true"/>
+    <col min="1" max="1" width="6.88671875" customWidth="true"/>
+    <col min="2" max="2" width="8.88671875" customWidth="true"/>
     <col min="3" max="3" width="5.33203125" customWidth="true"/>
     <col min="4" max="4" width="13.21875" customWidth="true"/>
     <col min="5" max="5" width="18" customWidth="true"/>
-    <col min="6" max="6" width="13.5546875" customWidth="true"/>
+    <col min="6" max="6" width="12.88671875" customWidth="true"/>
     <col min="7" max="7" width="14.5546875" customWidth="true"/>
     <col min="8" max="8" width="11.5546875" customWidth="true"/>
   </cols>
@@ -5342,16 +5345,16 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="0">
-        <v>25230</v>
+        <v>22150</v>
       </c>
       <c r="E2" s="0">
         <v>0</v>
@@ -5360,88 +5363,88 @@
         <v>0</v>
       </c>
       <c r="G2" s="0">
-        <v>504.60000000000002</v>
+        <v>443</v>
       </c>
       <c r="H2" s="0">
-        <v>502.60000000000002</v>
+        <v>440.80000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="0">
-        <v>25230</v>
+        <v>22150</v>
       </c>
       <c r="E3" s="0">
-        <v>0</v>
+        <v>290</v>
       </c>
       <c r="F3" s="0">
-        <v>0</v>
+        <v>1.3092550790067718</v>
       </c>
       <c r="G3" s="0">
-        <v>504.60000000000002</v>
+        <v>437.19999999999999</v>
       </c>
       <c r="H3" s="0">
-        <v>502.60000000000002</v>
+        <v>426.19999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="0">
-        <v>73750</v>
+        <v>1816140</v>
       </c>
       <c r="E4" s="0">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="F4" s="0">
-        <v>0.8677966101694915</v>
+        <v>0</v>
       </c>
       <c r="G4" s="0">
-        <v>1462.2</v>
+        <v>36322.800000000003</v>
       </c>
       <c r="H4" s="0">
-        <v>1416</v>
+        <v>36320.800000000003</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="0">
-        <v>73750</v>
+        <v>1816140</v>
       </c>
       <c r="E5" s="0">
-        <v>110</v>
+        <v>320</v>
       </c>
       <c r="F5" s="0">
-        <v>0.14915254237288136</v>
+        <v>0.017619787020824385</v>
       </c>
       <c r="G5" s="0">
-        <v>1472.8</v>
+        <v>36316.400000000001</v>
       </c>
       <c r="H5" s="0">
-        <v>1468.8</v>
+        <v>36309.199999999997</v>
       </c>
     </row>
     <row r="6">

</xml_diff>